<commit_message>
Refactor login automation framework and improve login validation
</commit_message>
<xml_diff>
--- a/data/LoginData.xlsx
+++ b/data/LoginData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\KTMB\KTMB_QA\Login Module\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC76568E-02D8-4900-A7A7-891D0612DE34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8963AD8-6B60-434F-A68E-5626E3B72E36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="750" windowWidth="29040" windowHeight="15720" xr2:uid="{955736AE-03FE-4685-8283-D767D114004E}"/>
+    <workbookView xWindow="29940" yWindow="2010" windowWidth="21600" windowHeight="11175" xr2:uid="{955736AE-03FE-4685-8283-D767D114004E}"/>
   </bookViews>
   <sheets>
     <sheet name="Login Data" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="23">
   <si>
     <t>TestCaseID</t>
   </si>
@@ -84,13 +84,37 @@
   </si>
   <si>
     <t>Abc123456</t>
+  </si>
+  <si>
+    <t>TC006</t>
+  </si>
+  <si>
+    <t>Validation</t>
+  </si>
+  <si>
+    <t>login_success</t>
+  </si>
+  <si>
+    <t>invalid_credential</t>
+  </si>
+  <si>
+    <t>invalid_email_format</t>
+  </si>
+  <si>
+    <t>empty_username</t>
+  </si>
+  <si>
+    <t>empty_password</t>
+  </si>
+  <si>
+    <t>multiple_login</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -110,6 +134,14 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -136,7 +168,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -145,6 +177,9 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -482,16 +517,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC42E17B-F5C7-4449-84DE-07B2509834E7}">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.7265625" customWidth="1"/>
     <col min="2" max="2" width="20.1796875" customWidth="1"/>
     <col min="3" max="3" width="15.1796875" customWidth="1"/>
     <col min="4" max="4" width="22.1796875" customWidth="1"/>
+    <col min="5" max="6" width="16.6328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -504,8 +540,11 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
+      <c r="E1" s="1" t="s">
+        <v>16</v>
+      </c>
     </row>
-    <row r="2" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
@@ -518,8 +557,11 @@
       <c r="D2" s="2" t="s">
         <v>6</v>
       </c>
+      <c r="E2" s="2" t="s">
+        <v>17</v>
+      </c>
     </row>
-    <row r="3" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>7</v>
       </c>
@@ -532,12 +574,15 @@
       <c r="D3" s="2" t="s">
         <v>9</v>
       </c>
+      <c r="E3" s="2" t="s">
+        <v>18</v>
+      </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="2" t="s">
         <v>14</v>
       </c>
       <c r="C4" s="2">
@@ -546,34 +591,63 @@
       <c r="D4" s="2" t="s">
         <v>9</v>
       </c>
+      <c r="E4" s="2" t="s">
+        <v>19</v>
+      </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="2"/>
+      <c r="B5" s="4"/>
       <c r="C5" s="2" t="s">
         <v>5</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>9</v>
       </c>
+      <c r="E5" s="2" t="s">
+        <v>20</v>
+      </c>
     </row>
-    <row r="6" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>12</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C6" s="2"/>
+      <c r="C6" s="4"/>
       <c r="D6" s="2" t="s">
         <v>9</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="A7" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>22</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B3" r:id="rId1" display="mailto:invalid@email.com" xr:uid="{2F1A7F1A-90F4-4B99-AA19-00637F13B94B}"/>
+    <hyperlink ref="B2" r:id="rId1" display="mailto:asyraaf.azman@gohub.com.my" xr:uid="{7B1C07B8-CE1C-4709-B9D5-B7B62A3A76E0}"/>
+    <hyperlink ref="B3" r:id="rId2" display="mailto:invalid@email.com" xr:uid="{B8F8EFBD-9D46-4079-ABC4-829B3F57C984}"/>
+    <hyperlink ref="B6" r:id="rId3" display="mailto:asyraaf.azman@gohub.com.my" xr:uid="{619587D1-6668-4508-B0FC-343A4D4AAFE7}"/>
+    <hyperlink ref="B7" r:id="rId4" display="mailto:asyraaf.azman@gohub.com.my" xr:uid="{70F80D6B-48E9-4693-A0A3-32DDBA6E80E7}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>